<commit_message>
Wrap all Excel calls in a structured error boundary; preserve VBA on .xlsm saves
- backends._excel_operation guards all 29 xlw_/com_ functions, turning opaque
  COM failures into ActionExecutionError while passing through the types the
  primitives contract raises deliberately (ValueError, NotImplementedError,
  FileNotFoundError, TimeoutError) so backend parity is unaffected
- test walks the module and fails if any xlw_/com_ function loses the guard
- cli.main gains a catch-all so no traceback can reach a user
- com_calculate_workbook delegates to com_calculate_sheet instead of repeating
  the raw Worksheet.Calculate call
- open_workbook sets keep_vba for macro-enabled formats only: without it an
  .xlsm silently loses xl/vbaProject.bin on save, with it unconditionally every
  .xlsx is mislabelled macroEnabled and Excel rejects it
- close_workbook releases the cached VBA archive openpyxl leaves dangling
</commit_message>
<xml_diff>
--- a/demos/08_full_showcase/linked_workbook/originals/linked.xlsx
+++ b/demos/08_full_showcase/linked_workbook/originals/linked.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\projects\excel-runner\demos\08_full_showcase\linked_workbook\originals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60FB0E67-1577-4C28-A399-F1C43774A8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50ABEDB2-F973-4442-AAAC-24AFBBC3F7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{21F20C5D-645B-4D95-96FD-A1C1FE82AF46}"/>
+    <workbookView xWindow="2820" yWindow="0" windowWidth="17280" windowHeight="8880" xr2:uid="{B315CC79-6F97-4969-8FF1-DA609378CC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,12 +41,26 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>Foo</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -102,11 +116,15 @@
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Products"/>
     </sheetNames>
+    <definedNames>
+      <definedName name="GrandTotalName" refersTo="='Products'!$F$2"/>
+    </definedNames>
     <sheetDataSet>
       <sheetData sheetId="0">
         <row r="2">
@@ -436,19 +454,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8411A5FF-893F-4571-BA0B-F6D8D68F0503}">
-  <dimension ref="A1:A3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99D307E5-0BD3-44CF-9B64-4D6C30B4056C}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1">
-        <f>[1]Products!F2</f>
+      <c r="A1" cm="1">
+        <f t="array" ref="A1">[1]!GrandTotalName</f>
         <v>322</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>